<commit_message>
Refactor, simplification, bug fixes, standarization, agent radius changed
</commit_message>
<xml_diff>
--- a/Metrics/SFM_Calibration_crossing.xlsx
+++ b/Metrics/SFM_Calibration_crossing.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Piotr\CrowdEvacuation\Metrics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CDAAC50-5F98-4D14-BF04-EF80F394C5E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF240559-D71C-44DB-B663-236EF34F9773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E00F018A-51B7-4FBE-B871-94FC33AFF981}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>#</t>
   </si>
@@ -77,9 +77,6 @@
     <t>Fine tuning:</t>
   </si>
   <si>
-    <t>Stałe:  m=80kg, r=0.2m, v₀=N(1.34,0.26) m/s</t>
-  </si>
-  <si>
     <t>KALIBRACJA SFM - Grid Search na Crossing_90 D_007</t>
   </si>
   <si>
@@ -164,19 +161,7 @@
     <t>Throughput (exit south) [p/s]</t>
   </si>
   <si>
-    <t>kanoniczny (inne r), zator nie pojawia się na środku skrzyżowania jak w ghost tylko w na południowo-wschodnim rogu skrzyżowania; agenci spychają się na niepożądane wyjścia po czym muszą wrócic z powrotem na swój korytarz</t>
-  </si>
-  <si>
-    <t>dochodzi do zderzen między agentami, nie wymijają się tak chętnie, symulacja nie wygląda naturlanie, ten sam zator co powyżej</t>
-  </si>
-  <si>
-    <t>nadal dochodzi do zderzeń i tego samego zatoru, agenci mniej agresywnie zmieniają swoją predkosc</t>
-  </si>
-  <si>
-    <t>trzymanie zauważalnie większych odstępów dzięki czemu nie dochodzi do kolizji, dochodzi jednak nadal do tego samego zatoru lecz nie przy samym rogu - jest to bardziej rozłożone; zostało kilku agentów na koniec którzy wolno wracali do swojego korytarza</t>
-  </si>
-  <si>
-    <t>dochodzi do zderzeń ale nie aż tak mocno jak w cal_01; pojawia się ten sam zator, ageci poruszają się szybciej, na koniec nie zostało wolno poruszających się agentów</t>
+    <t>Stałe:  m=80kg, r=N(0.23,0.01) m, v₀=N(1.34,0.26) m/s</t>
   </si>
 </sst>
 </file>
@@ -207,12 +192,14 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
+      <charset val="238"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
+      <charset val="238"/>
     </font>
     <font>
       <sz val="11"/>
@@ -250,7 +237,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -277,14 +264,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -327,7 +308,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -380,6 +361,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -389,19 +376,10 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -758,58 +736,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
+      <c r="N2" s="19"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
-    </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -833,11 +811,11 @@
       <c r="G5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="25" t="s">
+      <c r="H5" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="18" t="s">
         <v>40</v>
-      </c>
-      <c r="I5" s="25" t="s">
-        <v>41</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>5</v>
@@ -855,7 +833,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>1</v>
       </c>
@@ -874,33 +852,21 @@
       <c r="F6" s="13">
         <v>0.5</v>
       </c>
-      <c r="G6" s="5">
-        <v>157.82</v>
-      </c>
-      <c r="H6" s="5">
-        <v>2.14</v>
-      </c>
-      <c r="I6" s="5">
-        <v>1.7</v>
-      </c>
-      <c r="J6" s="5">
-        <v>0.92</v>
-      </c>
-      <c r="K6" s="7">
-        <v>0.69</v>
-      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="7"/>
       <c r="L6" s="6">
         <f>0.3*ABS(G6-134.12)/134.12 + 0.125*ABS(H6-2.07)/2.07 + 0.125*ABS(I6-2.44)/2.44 + 0.2*ABS(J6-0.53)/0.53 + 0.25*ABS(K6-0.5)/0.5</f>
-        <v>0.33731892838207678</v>
+        <v>1</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="N6" s="15" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+      <c r="N6" s="15"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>2</v>
       </c>
@@ -919,33 +885,21 @@
       <c r="F7" s="14">
         <v>0.3</v>
       </c>
-      <c r="G7" s="8">
-        <v>148.04</v>
-      </c>
-      <c r="H7" s="8">
-        <v>2</v>
-      </c>
-      <c r="I7" s="8">
-        <v>2.09</v>
-      </c>
-      <c r="J7" s="8">
-        <v>0.99</v>
-      </c>
-      <c r="K7" s="8">
-        <v>0.63</v>
-      </c>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
       <c r="L7" s="9">
         <f t="shared" ref="L7:L26" si="0">0.3*ABS(G7-134.12)/134.12 + 0.125*ABS(H7-2.07)/2.07 + 0.125*ABS(I7-2.44)/2.44 + 0.2*ABS(J7-0.53)/0.53 + 0.25*ABS(K7-0.5)/0.5</f>
-        <v>0.29187858252378507</v>
+        <v>1</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="N7" s="16" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+      <c r="N7" s="16"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>3</v>
       </c>
@@ -964,33 +918,21 @@
       <c r="F8" s="14">
         <v>0.5</v>
       </c>
-      <c r="G8" s="8">
-        <v>148.82</v>
-      </c>
-      <c r="H8" s="8">
-        <v>2.14</v>
-      </c>
-      <c r="I8" s="8">
-        <v>1.93</v>
-      </c>
-      <c r="J8" s="8">
-        <v>0.97</v>
-      </c>
-      <c r="K8" s="8">
-        <v>0.64</v>
-      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
       <c r="L8" s="9">
         <f t="shared" si="0"/>
-        <v>0.29927284025716372</v>
+        <v>1</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="N8" s="16" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+      <c r="N8" s="16"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>4</v>
       </c>
@@ -1009,33 +951,21 @@
       <c r="F9" s="14">
         <v>0.5</v>
       </c>
-      <c r="G9" s="11">
-        <v>158.30000000000001</v>
-      </c>
-      <c r="H9" s="11">
-        <v>2.02</v>
-      </c>
-      <c r="I9" s="11">
-        <v>1.81</v>
-      </c>
-      <c r="J9" s="11">
-        <v>0.88</v>
-      </c>
-      <c r="K9" s="11">
-        <v>0.72</v>
-      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
       <c r="L9" s="9">
         <f t="shared" si="0"/>
-        <v>0.33145527876348851</v>
+        <v>1</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="N9" s="16" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" ht="72" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+      <c r="N9" s="16"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>5</v>
       </c>
@@ -1054,31 +984,19 @@
       <c r="F10" s="14">
         <v>0.3</v>
       </c>
-      <c r="G10" s="8">
-        <v>150.66</v>
-      </c>
-      <c r="H10" s="8">
-        <v>1.92</v>
-      </c>
-      <c r="I10" s="8">
-        <v>2.1</v>
-      </c>
-      <c r="J10" s="8">
-        <v>1.01</v>
-      </c>
-      <c r="K10" s="8">
-        <v>0.65</v>
-      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
       <c r="L10" s="9">
         <f t="shared" si="0"/>
-        <v>0.31960479862887686</v>
+        <v>1</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="N10" s="16" t="s">
-        <v>46</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="N10" s="16"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -1109,7 +1027,7 @@
         <v>1</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N11" s="16"/>
     </row>
@@ -1142,7 +1060,7 @@
         <v>1</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="N12" s="16"/>
     </row>
@@ -1175,7 +1093,7 @@
         <v>1</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N13" s="16"/>
     </row>
@@ -1208,7 +1126,7 @@
         <v>1</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="N14" s="16"/>
     </row>
@@ -1241,7 +1159,7 @@
         <v>1</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="N15" s="16"/>
     </row>
@@ -1274,7 +1192,7 @@
         <v>1</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="N16" s="16"/>
     </row>
@@ -1307,7 +1225,7 @@
         <v>1</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="N17" s="16"/>
     </row>
@@ -1340,7 +1258,7 @@
         <v>1</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="N18" s="17"/>
     </row>
@@ -1373,7 +1291,7 @@
         <v>1</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N19" s="17"/>
     </row>
@@ -1406,42 +1324,42 @@
         <v>1</v>
       </c>
       <c r="M20" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="N20" s="17"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A21" s="20">
+        <v>16</v>
+      </c>
+      <c r="B21" s="21">
+        <v>800</v>
+      </c>
+      <c r="C21" s="21">
+        <v>0.08</v>
+      </c>
+      <c r="D21" s="21">
+        <v>60000</v>
+      </c>
+      <c r="E21" s="21">
+        <v>120000</v>
+      </c>
+      <c r="F21" s="21">
+        <v>0.3</v>
+      </c>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="9">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="M21" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="N20" s="17"/>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="18">
-        <v>16</v>
-      </c>
-      <c r="B21" s="19">
-        <v>800</v>
-      </c>
-      <c r="C21" s="19">
-        <v>0.08</v>
-      </c>
-      <c r="D21" s="19">
-        <v>60000</v>
-      </c>
-      <c r="E21" s="19">
-        <v>120000</v>
-      </c>
-      <c r="F21" s="19">
-        <v>0.3</v>
-      </c>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
-      <c r="J21" s="20"/>
-      <c r="K21" s="20"/>
-      <c r="L21" s="21">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-      <c r="M21" s="22" t="s">
-        <v>31</v>
-      </c>
-      <c r="N21" s="23"/>
+      <c r="N21" s="24"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
@@ -1472,7 +1390,7 @@
         <v>1</v>
       </c>
       <c r="M22" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="N22" s="17"/>
     </row>
@@ -1505,7 +1423,7 @@
         <v>1</v>
       </c>
       <c r="M23" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="N23" s="17"/>
     </row>
@@ -1538,7 +1456,7 @@
         <v>1</v>
       </c>
       <c r="M24" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="N24" s="17"/>
     </row>
@@ -1571,7 +1489,7 @@
         <v>1</v>
       </c>
       <c r="M25" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="N25" s="17"/>
     </row>
@@ -1604,27 +1522,27 @@
         <v>1</v>
       </c>
       <c r="M26" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N26" s="17"/>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A30" s="24" t="s">
+      <c r="A30" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="24"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="24"/>
-      <c r="I30" s="24"/>
-      <c r="J30" s="24"/>
-      <c r="K30" s="24"/>
-      <c r="L30" s="24"/>
-      <c r="M30" s="24"/>
-      <c r="N30" s="24"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="19"/>
+      <c r="F30" s="19"/>
+      <c r="G30" s="19"/>
+      <c r="H30" s="19"/>
+      <c r="I30" s="19"/>
+      <c r="J30" s="19"/>
+      <c r="K30" s="19"/>
+      <c r="L30" s="19"/>
+      <c r="M30" s="19"/>
+      <c r="N30" s="19"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
@@ -1645,7 +1563,7 @@
         <v>1</v>
       </c>
       <c r="M32" s="10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="N32" s="17"/>
     </row>
@@ -1668,7 +1586,7 @@
         <v>1</v>
       </c>
       <c r="M33" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="N33" s="17"/>
     </row>
@@ -1691,7 +1609,7 @@
         <v>1</v>
       </c>
       <c r="M34" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N34" s="17"/>
     </row>

</xml_diff>

<commit_message>
Improvements for crossing scene in training, bugfixes, agent spawning method changed
</commit_message>
<xml_diff>
--- a/Metrics/SFM_Calibration_crossing.xlsx
+++ b/Metrics/SFM_Calibration_crossing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Piotr\CrowdEvacuation\Metrics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{759E225B-4646-462E-8C22-342D35D02292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B65FE3E-5F10-47EE-93BE-0891F7C56A61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{E00F018A-51B7-4FBE-B871-94FC33AFF981}"/>
+    <workbookView xWindow="28680" yWindow="-180" windowWidth="29040" windowHeight="15720" xr2:uid="{E00F018A-51B7-4FBE-B871-94FC33AFF981}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="70">
   <si>
     <t>#</t>
   </si>
@@ -77,81 +77,6 @@
     <t>Fine tuning:</t>
   </si>
   <si>
-    <t>KALIBRACJA SFM - Grid Search na Crossing_90 D_007</t>
-  </si>
-  <si>
-    <t>D_007_SFM</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_01</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_02</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_03</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_04</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_05</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_06</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_07</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_08</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_09</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_10</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_11</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_12</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_13</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_14</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_15</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_16</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_17</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_18</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_19</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_20</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_21</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_22</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_23</t>
-  </si>
-  <si>
     <t>Throughput (exit west) [p/s]</t>
   </si>
   <si>
@@ -161,9 +86,6 @@
     <t>Stałe:  m=80kg, r=N(0.185,0.015) m, v₀=N(1.34,0.26) m/s</t>
   </si>
   <si>
-    <t>Cel empiryczny (Ghost D_007_SFM): RSET=133.69s, throughput (exit west)=2.08 ped/s, throughput (exit south)=2.45 ped/s, mean_speed=0.53 m/s, mean_headway=0,50 m</t>
-  </si>
-  <si>
     <t>kanoniczny z innym r - dobre wymijanie bez kolizji, zator tworzy się nie na środku (tak jak powinien) tylko na poludniowym zachodzie w rogu miedzy korytarzami, agenci sa wypychani nie na swój korytarz po czym musza wrocic do swojego</t>
   </si>
   <si>
@@ -188,12 +110,6 @@
     <t>ten sam przypadek jak powyżej lecz większe odbijanie się od siebie spowodowane mniejszym A i brakiem predykcji</t>
   </si>
   <si>
-    <t>pominięte - mniejsze A - gorszy wynik</t>
-  </si>
-  <si>
-    <t>---</t>
-  </si>
-  <si>
     <t>sprawniejsze przeciskanie w tłumie, lecz zator tworzy się znowu w tym samym miejscu zamiast na środku skrzyżowania</t>
   </si>
   <si>
@@ -230,15 +146,6 @@
     <t>utrzymywanie zacznie wiekszych odstepow co spowodowalo glowny zator na srodku, pojedynczy agenci nadal znalezli się w blednych korytarzach</t>
   </si>
   <si>
-    <t>D_007_SFM_cal_24</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_25</t>
-  </si>
-  <si>
-    <t>D_007_SFM_cal_26</t>
-  </si>
-  <si>
     <t>niekiedy zauważalne odpychanie między agentami, zator po czesci na srodku jednak grupują się też na rogu w nie tych korytarzach, dochodzi czasem do wpadania na siebie</t>
   </si>
   <si>
@@ -246,6 +153,99 @@
   </si>
   <si>
     <t>podobna sytuacja jak wyżej</t>
+  </si>
+  <si>
+    <t>mniejsze odległości między agentami, sprawneijsza ewakuacja -agenci nie stoją w korku jak w danych empirycznych</t>
+  </si>
+  <si>
+    <t>mniejsze odstępy, większy zator w rogu</t>
+  </si>
+  <si>
+    <t>KALIBRACJA SFM - Grid Search na Crossing_90 D_003</t>
+  </si>
+  <si>
+    <t>D_003_SFM</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_01</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_02</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_03</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_04</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_05</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_06</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_07</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_08</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_09</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_10</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_11</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_12</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_13</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_14</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_15</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_16</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_17</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_18</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_19</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_20</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_21</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_22</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_23</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_24</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_25</t>
+  </si>
+  <si>
+    <t>D_003_SFM_cal_26</t>
+  </si>
+  <si>
+    <t>Cel empiryczny (Ghost D_003_SFM): RSET=184s, throughput (exit west)=1.52 ped/s, throughput (exit south)=1.79 ped/s, mean_speed=1.02 m/s, mean_headway=0,61 m</t>
   </si>
 </sst>
 </file>
@@ -321,7 +321,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -356,12 +356,6 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -404,7 +398,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -475,29 +469,26 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -853,58 +844,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
+      <c r="A1" s="30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
+      <c r="K1" s="30"/>
+      <c r="L1" s="30"/>
+      <c r="M1" s="30"/>
+      <c r="N1" s="30"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24"/>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
+      <c r="A2" s="30" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-      <c r="L3" s="24"/>
-      <c r="M3" s="24"/>
-      <c r="N3" s="24"/>
+      <c r="A3" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+      <c r="J3" s="30"/>
+      <c r="K3" s="30"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="30"/>
+      <c r="N3" s="30"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
@@ -929,10 +920,10 @@
         <v>4</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="I5" s="18" t="s">
-        <v>39</v>
+        <v>14</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>5</v>
@@ -950,7 +941,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>1</v>
       </c>
@@ -969,30 +960,20 @@
       <c r="F6" s="13">
         <v>0.5</v>
       </c>
-      <c r="G6" s="5">
-        <v>146.63999999999999</v>
-      </c>
-      <c r="H6" s="5">
-        <v>2.2200000000000002</v>
-      </c>
-      <c r="I6" s="5">
-        <v>1.91</v>
-      </c>
-      <c r="J6" s="5">
-        <v>0.91</v>
-      </c>
-      <c r="K6" s="7">
-        <v>0.67</v>
-      </c>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="7"/>
       <c r="L6" s="6">
-        <f>0.15*ABS(G6-133.69)/133.69 + 0.1*ABS(H6-2.08)/2.08 + 0.1*ABS(I6-2.45)/2.45 + 0.35*ABS(J6-0.53)/0.53 + 0.3*ABS(K6-0.5)/0.5</f>
-        <v>0.39624486434785583</v>
+        <f>0.15*ABS(G6-184)/184 + 0.1*ABS(H6-1.52)/1.52 + 0.1*ABS(I6-1.79)/1.79 + 0.35*ABS(J6-1.02)/1.02 + 0.3*ABS(K6-0.61)/0.61</f>
+        <v>1</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="N6" s="15" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1014,30 +995,20 @@
       <c r="F7" s="14">
         <v>0.3</v>
       </c>
-      <c r="G7" s="8">
-        <v>145.69</v>
-      </c>
-      <c r="H7" s="8">
-        <v>2.09</v>
-      </c>
-      <c r="I7" s="8">
-        <v>2.0699999999999998</v>
-      </c>
-      <c r="J7" s="8">
-        <v>0.93</v>
-      </c>
-      <c r="K7" s="8">
-        <v>0.65</v>
-      </c>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
       <c r="L7" s="9">
-        <f t="shared" ref="L7:L27" si="0">0.15*ABS(G7-133.69)/133.69 + 0.1*ABS(H7-2.08)/2.08 + 0.1*ABS(I7-2.45)/2.45 + 0.35*ABS(J7-0.53)/0.53 + 0.3*ABS(K7-0.5)/0.5</f>
-        <v>0.38360590055184768</v>
+        <f t="shared" ref="L7:L27" si="0">0.15*ABS(G7-184)/184 + 0.1*ABS(H7-1.52)/1.52 + 0.1*ABS(I7-1.79)/1.79 + 0.35*ABS(J7-1.02)/1.02 + 0.3*ABS(K7-0.61)/0.61</f>
+        <v>1</v>
       </c>
       <c r="M7" s="10" t="s">
-        <v>15</v>
+        <v>43</v>
       </c>
       <c r="N7" s="16" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -1059,30 +1030,20 @@
       <c r="F8" s="14">
         <v>0.3</v>
       </c>
-      <c r="G8" s="8">
-        <v>146.18</v>
-      </c>
-      <c r="H8" s="8">
-        <v>1.98</v>
-      </c>
-      <c r="I8" s="8">
-        <v>2.16</v>
-      </c>
-      <c r="J8" s="8">
-        <v>0.97</v>
-      </c>
-      <c r="K8" s="8">
-        <v>0.64</v>
-      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
       <c r="L8" s="9">
         <f t="shared" si="0"/>
-        <v>0.40522422792090307</v>
+        <v>1</v>
       </c>
       <c r="M8" s="10" t="s">
-        <v>16</v>
+        <v>44</v>
       </c>
       <c r="N8" s="16" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -1104,30 +1065,20 @@
       <c r="F9" s="14">
         <v>0.3</v>
       </c>
-      <c r="G9" s="11">
-        <v>147.75</v>
-      </c>
-      <c r="H9" s="11">
-        <v>1.91</v>
-      </c>
-      <c r="I9" s="11">
-        <v>2.19</v>
-      </c>
-      <c r="J9" s="11">
-        <v>0.97</v>
-      </c>
-      <c r="K9" s="11">
-        <v>0.64</v>
-      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
       <c r="L9" s="9">
         <f t="shared" si="0"/>
-        <v>0.40912666062652386</v>
+        <v>1</v>
       </c>
       <c r="M9" s="10" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="N9" s="16" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1149,30 +1100,20 @@
       <c r="F10" s="14">
         <v>0.3</v>
       </c>
-      <c r="G10" s="8">
-        <v>150.69</v>
-      </c>
-      <c r="H10" s="8">
-        <v>1.84</v>
-      </c>
-      <c r="I10" s="8">
-        <v>2.1800000000000002</v>
-      </c>
-      <c r="J10" s="8">
-        <v>1.03</v>
-      </c>
-      <c r="K10" s="8">
-        <v>0.65</v>
-      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
       <c r="L10" s="9">
         <f t="shared" si="0"/>
-        <v>0.46182152605823734</v>
+        <v>1</v>
       </c>
       <c r="M10" s="10" t="s">
-        <v>18</v>
+        <v>46</v>
       </c>
       <c r="N10" s="16" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -1194,30 +1135,20 @@
       <c r="F11" s="14">
         <v>0.3</v>
       </c>
-      <c r="G11" s="8">
-        <v>152.74</v>
-      </c>
-      <c r="H11" s="8">
-        <v>1.83</v>
-      </c>
-      <c r="I11" s="8">
-        <v>2.13</v>
-      </c>
-      <c r="J11" s="8">
-        <v>1.03</v>
-      </c>
-      <c r="K11" s="8">
-        <v>0.62</v>
-      </c>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
       <c r="L11" s="9">
         <f t="shared" si="0"/>
-        <v>0.44864320885542047</v>
+        <v>1</v>
       </c>
       <c r="M11" s="10" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="72" x14ac:dyDescent="0.3">
@@ -1239,30 +1170,20 @@
       <c r="F12" s="14">
         <v>0.3</v>
       </c>
-      <c r="G12" s="8">
-        <v>149.65</v>
-      </c>
-      <c r="H12" s="8">
-        <v>1.95</v>
-      </c>
-      <c r="I12" s="8">
-        <v>2.1</v>
-      </c>
-      <c r="J12" s="8">
-        <v>0.97</v>
-      </c>
-      <c r="K12" s="8">
-        <v>0.64</v>
-      </c>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
       <c r="L12" s="9">
         <f t="shared" si="0"/>
-        <v>0.41300885053304509</v>
+        <v>1</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="N12" s="16" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
@@ -1284,33 +1205,23 @@
       <c r="F13" s="14">
         <v>0.3</v>
       </c>
-      <c r="G13" s="8">
-        <v>156.05000000000001</v>
-      </c>
-      <c r="H13" s="8">
-        <v>1.81</v>
-      </c>
-      <c r="I13" s="8">
-        <v>2.08</v>
-      </c>
-      <c r="J13" s="8">
-        <v>1.06</v>
-      </c>
-      <c r="K13" s="8">
-        <v>0.65</v>
-      </c>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
       <c r="L13" s="9">
         <f t="shared" si="0"/>
-        <v>0.49317069994162793</v>
+        <v>1</v>
       </c>
       <c r="M13" s="10" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A14" s="2">
         <v>9</v>
       </c>
@@ -1329,33 +1240,23 @@
       <c r="F14" s="14">
         <v>0.3</v>
       </c>
-      <c r="G14" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="H14" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="I14" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="J14" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="K14" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="L14" s="9" t="e">
+      <c r="G14" s="24"/>
+      <c r="H14" s="24"/>
+      <c r="I14" s="24"/>
+      <c r="J14" s="24"/>
+      <c r="K14" s="24"/>
+      <c r="L14" s="9">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>1</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="N14" s="16" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
         <v>10</v>
       </c>
@@ -1374,30 +1275,20 @@
       <c r="F15" s="14">
         <v>0.3</v>
       </c>
-      <c r="G15" s="11">
-        <v>148.47</v>
-      </c>
-      <c r="H15" s="11">
-        <v>1.92</v>
-      </c>
-      <c r="I15" s="11">
-        <v>2.16</v>
-      </c>
-      <c r="J15" s="11">
-        <v>0.97</v>
-      </c>
-      <c r="K15" s="11">
-        <v>0.63</v>
-      </c>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
       <c r="L15" s="9">
         <f t="shared" si="0"/>
-        <v>0.40467822022226613</v>
+        <v>1</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="N15" s="16" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
@@ -1419,30 +1310,20 @@
       <c r="F16" s="14">
         <v>0.3</v>
       </c>
-      <c r="G16" s="8">
-        <v>148.65</v>
-      </c>
-      <c r="H16" s="8">
-        <v>1.87</v>
-      </c>
-      <c r="I16" s="8">
-        <v>2.21</v>
-      </c>
-      <c r="J16" s="8">
-        <v>1.04</v>
-      </c>
-      <c r="K16" s="8">
-        <v>0.65</v>
-      </c>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
       <c r="L16" s="9">
         <f t="shared" si="0"/>
-        <v>0.46346962490156968</v>
+        <v>1</v>
       </c>
       <c r="M16" s="10" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="N16" s="16" t="s">
-        <v>53</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
@@ -1464,30 +1345,20 @@
       <c r="F17" s="14">
         <v>0.3</v>
       </c>
-      <c r="G17" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="H17" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="I17" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="J17" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="K17" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="L17" s="9" t="e">
+      <c r="G17" s="24"/>
+      <c r="H17" s="24"/>
+      <c r="I17" s="24"/>
+      <c r="J17" s="24"/>
+      <c r="K17" s="24"/>
+      <c r="L17" s="9">
         <f t="shared" si="0"/>
-        <v>#VALUE!</v>
+        <v>1</v>
       </c>
       <c r="M17" s="10" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
       <c r="N17" s="16" t="s">
-        <v>50</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -1509,30 +1380,20 @@
       <c r="F18" s="20">
         <v>0.3</v>
       </c>
-      <c r="G18" s="3">
-        <v>148.11000000000001</v>
-      </c>
-      <c r="H18" s="3">
-        <v>1.99</v>
-      </c>
-      <c r="I18" s="3">
-        <v>2.1</v>
-      </c>
-      <c r="J18" s="3">
-        <v>0.94</v>
-      </c>
-      <c r="K18" s="3">
-        <v>0.65</v>
-      </c>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
       <c r="L18" s="9">
         <f t="shared" si="0"/>
-        <v>0.39554657492870471</v>
+        <v>1</v>
       </c>
       <c r="M18" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="N18" s="17" t="s">
         <v>26</v>
-      </c>
-      <c r="N18" s="17" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1554,30 +1415,20 @@
       <c r="F19" s="14">
         <v>0.3</v>
       </c>
-      <c r="G19" s="3">
-        <v>148.91999999999999</v>
-      </c>
-      <c r="H19" s="3">
-        <v>1.91</v>
-      </c>
-      <c r="I19" s="3">
-        <v>2.16</v>
-      </c>
-      <c r="J19" s="3">
-        <v>0.95</v>
-      </c>
-      <c r="K19" s="3">
-        <v>0.66</v>
-      </c>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
       <c r="L19" s="9">
         <f t="shared" si="0"/>
-        <v>0.41045634167734479</v>
+        <v>1</v>
       </c>
       <c r="M19" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="N19" s="17" t="s">
         <v>27</v>
-      </c>
-      <c r="N19" s="17" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -1599,30 +1450,20 @@
       <c r="F20" s="14">
         <v>0.3</v>
       </c>
-      <c r="G20" s="11">
-        <v>155.87</v>
-      </c>
-      <c r="H20" s="11">
-        <v>1.83</v>
-      </c>
-      <c r="I20" s="11">
-        <v>2.06</v>
-      </c>
-      <c r="J20" s="11">
-        <v>0.95</v>
-      </c>
-      <c r="K20" s="11">
-        <v>0.7</v>
-      </c>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
       <c r="L20" s="9">
         <f t="shared" si="0"/>
-        <v>0.45018201881909103</v>
+        <v>1</v>
       </c>
       <c r="M20" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="N20" s="17" t="s">
         <v>28</v>
-      </c>
-      <c r="N20" s="17" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1644,30 +1485,20 @@
       <c r="F21" s="20">
         <v>0.3</v>
       </c>
-      <c r="G21" s="21">
-        <v>147.31</v>
-      </c>
-      <c r="H21" s="21">
-        <v>2.0499999999999998</v>
-      </c>
-      <c r="I21" s="21">
-        <v>2.06</v>
-      </c>
-      <c r="J21" s="21">
-        <v>0.9</v>
-      </c>
-      <c r="K21" s="21">
-        <v>0.68</v>
-      </c>
+      <c r="G21" s="21"/>
+      <c r="H21" s="21"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="21"/>
+      <c r="K21" s="21"/>
       <c r="L21" s="9">
         <f t="shared" si="0"/>
-        <v>0.38498191934280995</v>
+        <v>1</v>
       </c>
       <c r="M21" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="N21" s="23" t="s">
         <v>29</v>
-      </c>
-      <c r="N21" s="23" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -1689,30 +1520,20 @@
       <c r="F22" s="14">
         <v>0.3</v>
       </c>
-      <c r="G22" s="3">
-        <v>147.38999999999999</v>
-      </c>
-      <c r="H22" s="3">
-        <v>1.95</v>
-      </c>
-      <c r="I22" s="3">
-        <v>2.16</v>
-      </c>
-      <c r="J22" s="3">
-        <v>0.95</v>
-      </c>
-      <c r="K22" s="3">
-        <v>0.73</v>
-      </c>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
       <c r="L22" s="9">
         <f t="shared" si="0"/>
-        <v>0.44881660681425739</v>
+        <v>1</v>
       </c>
       <c r="M22" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="N22" s="17" t="s">
         <v>30</v>
-      </c>
-      <c r="N22" s="17" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1734,30 +1555,20 @@
       <c r="F23" s="14">
         <v>0.3</v>
       </c>
-      <c r="G23" s="3">
-        <v>145.53</v>
-      </c>
-      <c r="H23" s="3">
-        <v>2.06</v>
-      </c>
-      <c r="I23" s="3">
-        <v>2.1</v>
-      </c>
-      <c r="J23" s="3">
-        <v>0.91</v>
-      </c>
-      <c r="K23" s="3">
-        <v>0.71</v>
-      </c>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
       <c r="L23" s="9">
         <f t="shared" si="0"/>
-        <v>0.40547511303231087</v>
+        <v>1</v>
       </c>
       <c r="M23" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="N23" s="17" t="s">
         <v>31</v>
-      </c>
-      <c r="N23" s="17" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -1779,30 +1590,20 @@
       <c r="F24" s="14">
         <v>0.5</v>
       </c>
-      <c r="G24" s="3">
-        <v>148.46</v>
-      </c>
-      <c r="H24" s="3">
-        <v>1.95</v>
-      </c>
-      <c r="I24" s="3">
-        <v>2.13</v>
-      </c>
-      <c r="J24" s="3">
-        <v>0.87</v>
-      </c>
-      <c r="K24" s="3">
-        <v>0.62</v>
-      </c>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
       <c r="L24" s="9">
         <f t="shared" si="0"/>
-        <v>0.3324114464902842</v>
+        <v>1</v>
       </c>
       <c r="M24" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="N24" s="17" t="s">
         <v>32</v>
-      </c>
-      <c r="N24" s="17" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
@@ -1824,78 +1625,58 @@
       <c r="F25" s="14">
         <v>0.5</v>
       </c>
-      <c r="G25" s="3">
-        <v>149.87</v>
-      </c>
-      <c r="H25" s="3">
-        <v>1.91</v>
-      </c>
-      <c r="I25" s="3">
-        <v>2.14</v>
-      </c>
-      <c r="J25" s="3">
-        <v>0.89</v>
-      </c>
-      <c r="K25" s="3">
-        <v>0.61</v>
-      </c>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
       <c r="L25" s="9">
         <f t="shared" si="0"/>
-        <v>0.34271592541944468</v>
+        <v>1</v>
       </c>
       <c r="M25" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="N25" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="N25" s="17" t="s">
-        <v>61</v>
-      </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="26">
+      <c r="A26" s="25">
         <v>21</v>
       </c>
-      <c r="B26" s="27">
+      <c r="B26" s="26">
         <v>800</v>
       </c>
-      <c r="C26" s="27">
+      <c r="C26" s="26">
         <v>0.12</v>
       </c>
-      <c r="D26" s="27">
+      <c r="D26" s="26">
         <v>80000</v>
       </c>
-      <c r="E26" s="27">
+      <c r="E26" s="26">
         <v>160000</v>
       </c>
-      <c r="F26" s="27">
+      <c r="F26" s="26">
         <v>0.5</v>
       </c>
-      <c r="G26" s="28">
-        <v>147.82</v>
-      </c>
-      <c r="H26" s="28">
-        <v>2.0499999999999998</v>
-      </c>
-      <c r="I26" s="28">
-        <v>2.0499999999999998</v>
-      </c>
-      <c r="J26" s="28">
-        <v>0.87</v>
-      </c>
-      <c r="K26" s="28">
-        <v>0.66</v>
-      </c>
-      <c r="L26" s="29">
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="9">
         <f t="shared" si="0"/>
-        <v>0.35415098116673588</v>
-      </c>
-      <c r="M26" s="30" t="s">
+        <v>1</v>
+      </c>
+      <c r="M26" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="N26" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="N26" s="31" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="27" spans="1:14" ht="77.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>22</v>
       </c>
@@ -1914,49 +1695,39 @@
       <c r="F27" s="14">
         <v>0.3</v>
       </c>
-      <c r="G27" s="3">
-        <v>153.68</v>
-      </c>
-      <c r="H27" s="3">
-        <v>2.02</v>
-      </c>
-      <c r="I27" s="3">
-        <v>1.93</v>
-      </c>
-      <c r="J27" s="3">
-        <v>0.89</v>
-      </c>
-      <c r="K27" s="3">
-        <v>0.8</v>
-      </c>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
       <c r="L27" s="9">
         <f t="shared" si="0"/>
-        <v>0.46427370732263384</v>
+        <v>1</v>
       </c>
       <c r="M27" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="N27" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="N27" s="17" t="s">
-        <v>63</v>
-      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="24" t="s">
+      <c r="A29" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="B29" s="24"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="24"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
-      <c r="K29" s="24"/>
-      <c r="L29" s="24"/>
-      <c r="M29" s="24"/>
-      <c r="N29" s="24"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="30"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="30"/>
     </row>
     <row r="31" spans="1:14" ht="72" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
@@ -1977,30 +1748,20 @@
       <c r="F31" s="14">
         <v>0.5</v>
       </c>
-      <c r="G31" s="3">
-        <v>147.75</v>
-      </c>
-      <c r="H31" s="3">
-        <v>2.25</v>
-      </c>
-      <c r="I31" s="3">
-        <v>1.85</v>
-      </c>
-      <c r="J31" s="3">
-        <v>0.88</v>
-      </c>
-      <c r="K31" s="3">
-        <v>0.69</v>
-      </c>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
       <c r="L31" s="9">
-        <f>0.15*ABS(G31-133.69)/133.69 + 0.1*ABS(H31-2.08)/2.08 + 0.1*ABS(I31-2.45)/2.45 + 0.35*ABS(J31-0.53)/0.53 + 0.3*ABS(K31-0.5)/0.5</f>
-        <v>0.39357024938278107</v>
+        <f>0.15*ABS(G31-184)/184 + 0.1*ABS(H31-1.52)/1.52 + 0.1*ABS(I31-1.79)/1.79 + 0.35*ABS(J31-1.02)/1.02 + 0.3*ABS(K31-0.61)/0.61</f>
+        <v>1</v>
       </c>
       <c r="M31" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="N31" s="17" t="s">
         <v>36</v>
-      </c>
-      <c r="N31" s="17" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
@@ -2022,30 +1783,20 @@
       <c r="F32" s="14">
         <v>0.5</v>
       </c>
-      <c r="G32" s="3">
-        <v>147.62</v>
-      </c>
-      <c r="H32" s="3">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="I32" s="3">
-        <v>1.9</v>
-      </c>
-      <c r="J32" s="3">
-        <v>0.88</v>
-      </c>
-      <c r="K32" s="3">
-        <v>0.74</v>
-      </c>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
       <c r="L32" s="9">
-        <f t="shared" ref="L32:L35" si="1">0.15*ABS(G32-133.69)/133.69 + 0.1*ABS(H32-2.08)/2.08 + 0.1*ABS(I32-2.45)/2.45 + 0.35*ABS(J32-0.53)/0.53 + 0.3*ABS(K32-0.5)/0.5</f>
-        <v>0.41897972707743614</v>
+        <f t="shared" ref="L32:L35" si="1">0.15*ABS(G32-184)/184 + 0.1*ABS(H32-1.52)/1.52 + 0.1*ABS(I32-1.79)/1.79 + 0.35*ABS(J32-1.02)/1.02 + 0.3*ABS(K32-0.61)/0.61</f>
+        <v>1</v>
       </c>
       <c r="M32" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="N32" s="17" t="s">
         <v>37</v>
-      </c>
-      <c r="N32" s="17" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
@@ -2067,30 +1818,20 @@
       <c r="F33" s="14">
         <v>0.5</v>
       </c>
-      <c r="G33" s="3">
-        <v>149.6</v>
-      </c>
-      <c r="H33" s="3">
-        <v>2.13</v>
-      </c>
-      <c r="I33" s="3">
-        <v>1.92</v>
-      </c>
-      <c r="J33" s="3">
-        <v>0.86</v>
-      </c>
-      <c r="K33" s="3">
-        <v>0.78</v>
-      </c>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
       <c r="L33" s="9">
         <f t="shared" si="1"/>
-        <v>0.42781202609575908</v>
+        <v>1</v>
       </c>
       <c r="M33" s="10" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="N33" s="17" t="s">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
@@ -2112,30 +1853,20 @@
       <c r="F34" s="14">
         <v>0.5</v>
       </c>
-      <c r="G34" s="3">
-        <v>148.93</v>
-      </c>
-      <c r="H34" s="3">
-        <v>2.2400000000000002</v>
-      </c>
-      <c r="I34" s="3">
-        <v>1.83</v>
-      </c>
-      <c r="J34" s="3">
-        <v>0.88</v>
-      </c>
-      <c r="K34" s="3">
-        <v>0.73</v>
-      </c>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
       <c r="L34" s="9">
         <f t="shared" si="1"/>
-        <v>0.419229765093874</v>
+        <v>1</v>
       </c>
       <c r="M34" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="N34" s="17" t="s">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
@@ -2157,30 +1888,20 @@
       <c r="F35" s="14">
         <v>0.5</v>
       </c>
-      <c r="G35" s="3">
-        <v>149.09</v>
-      </c>
-      <c r="H35" s="3">
-        <v>2.1</v>
-      </c>
-      <c r="I35" s="3">
-        <v>1.97</v>
-      </c>
-      <c r="J35" s="3">
-        <v>0.88</v>
-      </c>
-      <c r="K35" s="3">
-        <v>0.79</v>
-      </c>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
       <c r="L35" s="9">
         <f t="shared" si="1"/>
-        <v>0.44296422993339535</v>
+        <v>1</v>
       </c>
       <c r="M35" s="10" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="N35" s="17" t="s">
-        <v>69</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>